<commit_message>
Update analyzer to include krd calculations
</commit_message>
<xml_diff>
--- a/Excel tester.xlsx
+++ b/Excel tester.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mariakantardjian/Desktop/Fixed-Income Yield Curve Sensitivity Analyzer/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mariakantardjian/Desktop/yield-curve-analyzer/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30A488C0-BACE-C34D-B2C7-2FF02E2533E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CC9EBE6-1BA3-E741-8244-A20D61E65DE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16940" xr2:uid="{A28DB794-6771-3841-A121-910A7CFF0B87}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
   <si>
     <t>Tenor</t>
   </si>
@@ -72,6 +72,21 @@
   </si>
   <si>
     <t>shocks:</t>
+  </si>
+  <si>
+    <t>PV0</t>
+  </si>
+  <si>
+    <t>PV+</t>
+  </si>
+  <si>
+    <t>PV-</t>
+  </si>
+  <si>
+    <t>Duration</t>
+  </si>
+  <si>
+    <t>2yr shock</t>
   </si>
 </sst>
 </file>
@@ -495,13 +510,15 @@
   <cols>
     <col min="1" max="1" width="7.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="8" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.1640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.83203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.1640625" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="8" bestFit="1" customWidth="1"/>
-    <col min="10" max="13" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="5.6640625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="8.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -733,11 +750,11 @@
         <v>4.65E-2</v>
       </c>
       <c r="F15" s="5">
-        <f t="shared" ref="F15:F24" si="0">$B$16*$B$18</f>
+        <f t="shared" ref="F15:F23" si="0">$B$16*$B$18</f>
         <v>50</v>
       </c>
       <c r="G15" s="6">
-        <f>F15/(1+E15)^D15</f>
+        <f t="shared" ref="G15:G24" si="1">F15/(1+E15)^D15</f>
         <v>47.778308647873864</v>
       </c>
       <c r="I15" s="2"/>
@@ -755,7 +772,7 @@
         <v>0.05</v>
       </c>
       <c r="D16" s="7">
-        <f>D15+1</f>
+        <f t="shared" ref="D16:D24" si="2">D15+1</f>
         <v>2</v>
       </c>
       <c r="E16" s="8">
@@ -766,12 +783,12 @@
         <v>50</v>
       </c>
       <c r="G16" s="6">
-        <f>F16/(1+E16)^D16</f>
+        <f t="shared" si="1"/>
         <v>45.611740097007058</v>
       </c>
       <c r="I16" s="2"/>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>0</v>
       </c>
@@ -779,7 +796,7 @@
         <v>10</v>
       </c>
       <c r="D17" s="7">
-        <f>D16+1</f>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="E17" s="8">
@@ -790,12 +807,15 @@
         <v>50</v>
       </c>
       <c r="G17" s="6">
-        <f>F17/(1+E17)^D17</f>
+        <f t="shared" si="1"/>
         <v>43.501868316881023</v>
       </c>
       <c r="I17" s="2"/>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="K17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>3</v>
       </c>
@@ -803,7 +823,7 @@
         <v>1000</v>
       </c>
       <c r="D18" s="7">
-        <f>D17+1</f>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="E18" s="8">
@@ -815,17 +835,23 @@
         <v>50</v>
       </c>
       <c r="G18" s="6">
-        <f>F18/(1+E18)^D18</f>
+        <f t="shared" si="1"/>
         <v>41.489607497793237</v>
       </c>
       <c r="I18" s="2"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="K18" s="1">
+        <v>1008.17</v>
+      </c>
+      <c r="L18" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>4</v>
       </c>
       <c r="D19" s="7">
-        <f>D18+1</f>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
       <c r="E19" s="8">
@@ -836,14 +862,20 @@
         <v>50</v>
       </c>
       <c r="G19" s="6">
-        <f>F19/(1+E19)^D19</f>
+        <f t="shared" si="1"/>
         <v>39.551557577704969</v>
       </c>
       <c r="I19" s="2"/>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="K19" s="1">
+        <v>1009.92</v>
+      </c>
+      <c r="L19" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="D20" s="7">
-        <f>D19+1</f>
+        <f t="shared" si="2"/>
         <v>6</v>
       </c>
       <c r="E20" s="8">
@@ -855,14 +887,20 @@
         <v>50</v>
       </c>
       <c r="G20" s="6">
-        <f>F20/(1+E20)^D20</f>
+        <f t="shared" si="1"/>
         <v>37.686063701281441</v>
       </c>
       <c r="I20" s="2"/>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="K20" s="1">
+        <v>1009.03</v>
+      </c>
+      <c r="L20" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="D21" s="7">
-        <f>D20+1</f>
+        <f t="shared" si="2"/>
         <v>7</v>
       </c>
       <c r="E21" s="8">
@@ -873,13 +911,20 @@
         <v>50</v>
       </c>
       <c r="G21" s="6">
-        <f>F21/(1+E21)^D21</f>
+        <f t="shared" si="1"/>
         <v>35.891446423054923</v>
       </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="K21">
+        <f>(K19-K18)/(2*0.01*K20)</f>
+        <v>8.6716945977820287E-2</v>
+      </c>
+      <c r="L21" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="D22" s="7">
-        <f>D21+1</f>
+        <f t="shared" si="2"/>
         <v>8</v>
       </c>
       <c r="E22" s="8">
@@ -891,13 +936,13 @@
         <v>50</v>
       </c>
       <c r="G22" s="6">
-        <f>F22/(1+E22)^D22</f>
+        <f t="shared" si="1"/>
         <v>34.187732390394075</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="D23" s="7">
-        <f>D22+1</f>
+        <f t="shared" si="2"/>
         <v>9</v>
       </c>
       <c r="E23" s="8">
@@ -909,13 +954,13 @@
         <v>50</v>
       </c>
       <c r="G23" s="6">
-        <f>F23/(1+E23)^D23</f>
+        <f t="shared" si="1"/>
         <v>32.554548168665434</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="D24" s="7">
-        <f>D23+1</f>
+        <f t="shared" si="2"/>
         <v>10</v>
       </c>
       <c r="E24" s="8">
@@ -926,11 +971,11 @@
         <v>1050</v>
       </c>
       <c r="G24" s="6">
-        <f>F24/(1+E24)^D24</f>
+        <f t="shared" si="1"/>
         <v>650.78032899853008</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="D25" s="7"/>
       <c r="E25" s="8"/>
       <c r="F25" s="5"/>

</xml_diff>